<commit_message>
#174 Updated parts Highlighted in BOM
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Top_Board_v3.5/BOM/Client_BOM_LSS_Top_Board_v3.5.xlsx
+++ b/Design-Files/LSS_Top_Board_v3.5/BOM/Client_BOM_LSS_Top_Board_v3.5.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="405">
   <si>
     <t>#</t>
   </si>
@@ -1225,6 +1225,15 @@
   </si>
   <si>
     <t>Bivar Inc.</t>
+  </si>
+  <si>
+    <t>Addition R11, R22, R25, R27</t>
+  </si>
+  <si>
+    <t>0603WAF1201T5E</t>
+  </si>
+  <si>
+    <t>RTT03R330FTP</t>
   </si>
 </sst>
 </file>
@@ -1308,7 +1317,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1324,6 +1333,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1437,7 +1452,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1474,9 +1489,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1493,6 +1505,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1796,6 +1823,8 @@
     <col min="9" max="9" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.85546875" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1807,9 +1836,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1906,7 +1935,7 @@
       <c r="J4" s="9">
         <v>11</v>
       </c>
-      <c r="K4" s="15" t="s">
+      <c r="K4" s="14" t="s">
         <v>385</v>
       </c>
     </row>
@@ -2132,7 +2161,7 @@
       <c r="J11" s="7">
         <v>8</v>
       </c>
-      <c r="K11" s="15" t="s">
+      <c r="K11" s="14" t="s">
         <v>394</v>
       </c>
     </row>
@@ -2465,28 +2494,28 @@
       <c r="C22" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="G22" s="22" t="s">
         <v>253</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="21" t="s">
         <v>294</v>
       </c>
-      <c r="I22" s="10" t="s">
+      <c r="I22" s="22" t="s">
         <v>337</v>
       </c>
-      <c r="J22" s="9">
+      <c r="J22" s="21">
         <v>3</v>
       </c>
-      <c r="K22" s="9"/>
+      <c r="K22" s="21"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
@@ -2849,28 +2878,28 @@
       <c r="C34" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="D34" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="E34" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="F34" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="G34" s="10" t="s">
+      <c r="G34" s="22" t="s">
         <v>261</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="21" t="s">
         <v>308</v>
       </c>
-      <c r="I34" s="8" t="s">
+      <c r="I34" s="23" t="s">
         <v>396</v>
       </c>
-      <c r="J34" s="9">
-        <v>1</v>
-      </c>
-      <c r="K34" s="9"/>
+      <c r="J34" s="21">
+        <v>1</v>
+      </c>
+      <c r="K34" s="21"/>
     </row>
     <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
@@ -2881,28 +2910,28 @@
       <c r="C35" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E35" s="8" t="s">
+      <c r="E35" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="F35" s="24" t="s">
         <v>205</v>
       </c>
-      <c r="G35" s="8" t="s">
+      <c r="G35" s="23" t="s">
         <v>262</v>
       </c>
-      <c r="H35" s="7" t="s">
+      <c r="H35" s="24" t="s">
         <v>309</v>
       </c>
-      <c r="I35" s="8" t="s">
+      <c r="I35" s="23" t="s">
         <v>396</v>
       </c>
-      <c r="J35" s="7">
-        <v>1</v>
-      </c>
-      <c r="K35" s="7"/>
+      <c r="J35" s="24">
+        <v>1</v>
+      </c>
+      <c r="K35" s="24"/>
     </row>
     <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
@@ -2913,28 +2942,28 @@
       <c r="C36" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="E36" s="10" t="s">
+      <c r="E36" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="F36" s="9" t="s">
+      <c r="F36" s="21" t="s">
         <v>206</v>
       </c>
-      <c r="G36" s="10" t="s">
+      <c r="G36" s="22" t="s">
         <v>263</v>
       </c>
-      <c r="H36" s="9" t="s">
+      <c r="H36" s="21" t="s">
         <v>310</v>
       </c>
-      <c r="I36" s="8" t="s">
+      <c r="I36" s="23" t="s">
         <v>396</v>
       </c>
-      <c r="J36" s="9">
-        <v>1</v>
-      </c>
-      <c r="K36" s="9"/>
+      <c r="J36" s="21">
+        <v>1</v>
+      </c>
+      <c r="K36" s="21"/>
     </row>
     <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
@@ -2945,28 +2974,28 @@
       <c r="C37" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="E37" s="8" t="s">
+      <c r="E37" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="F37" s="7" t="s">
+      <c r="F37" s="24" t="s">
         <v>207</v>
       </c>
-      <c r="G37" s="8" t="s">
+      <c r="G37" s="23" t="s">
         <v>264</v>
       </c>
-      <c r="H37" s="7" t="s">
+      <c r="H37" s="24" t="s">
         <v>311</v>
       </c>
-      <c r="I37" s="8" t="s">
+      <c r="I37" s="23" t="s">
         <v>396</v>
       </c>
-      <c r="J37" s="7">
+      <c r="J37" s="24">
         <v>2</v>
       </c>
-      <c r="K37" s="7"/>
+      <c r="K37" s="24"/>
     </row>
     <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
@@ -3099,28 +3128,28 @@
       <c r="C42" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D42" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E42" s="10" t="s">
+      <c r="E42" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="F42" s="9" t="s">
+      <c r="F42" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="G42" s="10" t="s">
+      <c r="G42" s="22" t="s">
         <v>266</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="H42" s="21" t="s">
         <v>313</v>
       </c>
-      <c r="I42" s="8" t="s">
+      <c r="I42" s="23" t="s">
         <v>396</v>
       </c>
-      <c r="J42" s="9">
-        <v>1</v>
-      </c>
-      <c r="K42" s="9"/>
+      <c r="J42" s="21">
+        <v>1</v>
+      </c>
+      <c r="K42" s="21"/>
     </row>
     <row r="43" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
@@ -3504,7 +3533,7 @@
       <c r="J54" s="9">
         <v>2</v>
       </c>
-      <c r="K54" s="16" t="s">
+      <c r="K54" s="15" t="s">
         <v>395</v>
       </c>
     </row>
@@ -3514,31 +3543,31 @@
         <f>ROW(B55) - ROW($B$2)</f>
         <v>53</v>
       </c>
-      <c r="C55" s="18" t="s">
+      <c r="C55" s="17" t="s">
         <v>360</v>
       </c>
-      <c r="D55" s="19" t="s">
+      <c r="D55" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="E55" s="20" t="s">
+      <c r="E55" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="F55" s="19" t="s">
+      <c r="F55" s="18" t="s">
         <v>396</v>
       </c>
-      <c r="G55" s="19" t="s">
+      <c r="G55" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="H55" s="19" t="s">
+      <c r="H55" s="18" t="s">
         <v>396</v>
       </c>
-      <c r="I55" s="20" t="s">
+      <c r="I55" s="19" t="s">
         <v>396</v>
       </c>
-      <c r="J55" s="19">
+      <c r="J55" s="18">
         <v>4</v>
       </c>
-      <c r="K55" s="19"/>
+      <c r="K55" s="18"/>
     </row>
     <row r="56" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
@@ -3581,28 +3610,28 @@
       <c r="C57" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D57" s="7" t="s">
+      <c r="D57" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="E57" s="8" t="s">
+      <c r="E57" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="F57" s="24" t="s">
         <v>223</v>
       </c>
-      <c r="G57" s="8" t="s">
+      <c r="G57" s="23" t="s">
         <v>268</v>
       </c>
-      <c r="H57" s="7" t="s">
+      <c r="H57" s="24" t="s">
         <v>322</v>
       </c>
-      <c r="I57" s="8" t="s">
+      <c r="I57" s="23" t="s">
         <v>396</v>
       </c>
-      <c r="J57" s="7">
-        <v>1</v>
-      </c>
-      <c r="K57" s="7"/>
+      <c r="J57" s="24">
+        <v>1</v>
+      </c>
+      <c r="K57" s="24"/>
     </row>
     <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
@@ -3730,7 +3759,9 @@
       <c r="J61" s="7">
         <v>6</v>
       </c>
-      <c r="K61" s="7"/>
+      <c r="K61" s="24" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
@@ -3933,28 +3964,28 @@
       <c r="C68" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D68" s="9" t="s">
+      <c r="D68" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="E68" s="10" t="s">
+      <c r="E68" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="F68" s="9" t="s">
+      <c r="F68" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="G68" s="10" t="s">
+      <c r="G68" s="22" t="s">
         <v>279</v>
       </c>
-      <c r="H68" s="9" t="s">
+      <c r="H68" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="I68" s="10" t="s">
+      <c r="I68" s="22" t="s">
         <v>371</v>
       </c>
-      <c r="J68" s="9">
-        <v>1</v>
-      </c>
-      <c r="K68" s="9"/>
+      <c r="J68" s="21">
+        <v>1</v>
+      </c>
+      <c r="K68" s="21"/>
     </row>
     <row r="69" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
@@ -4230,7 +4261,9 @@
       <c r="F77" s="7" t="s">
         <v>224</v>
       </c>
-      <c r="G77" s="8"/>
+      <c r="G77" s="8" t="s">
+        <v>403</v>
+      </c>
       <c r="H77" s="7" t="s">
         <v>324</v>
       </c>
@@ -4260,7 +4293,9 @@
       <c r="F78" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="G78" s="10"/>
+      <c r="G78" s="10" t="s">
+        <v>404</v>
+      </c>
       <c r="H78" s="9" t="s">
         <v>325</v>
       </c>
@@ -4649,7 +4684,7 @@
       <c r="J90" s="7">
         <v>1</v>
       </c>
-      <c r="K90" s="17"/>
+      <c r="K90" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
#174 BOM highlights edite
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Top_Board_v3.5/BOM/Client_BOM_LSS_Top_Board_v3.5.xlsx
+++ b/Design-Files/LSS_Top_Board_v3.5/BOM/Client_BOM_LSS_Top_Board_v3.5.xlsx
@@ -243,9 +243,6 @@
     <t>R4</t>
   </si>
   <si>
-    <t>R5, R11, R22, R25, R27, R32</t>
-  </si>
-  <si>
     <t>R6, R7, R8, R9</t>
   </si>
   <si>
@@ -1227,20 +1224,44 @@
     <t>Bivar Inc.</t>
   </si>
   <si>
-    <t>Addition R11, R22, R25, R27</t>
-  </si>
-  <si>
     <t>0603WAF1201T5E</t>
   </si>
   <si>
     <t>RTT03R330FTP</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">R5, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>R11, R22, R25, R27</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, R32</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Addition Highlighted with RED </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1310,6 +1331,21 @@
     </font>
     <font>
       <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1452,7 +1488,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1507,9 +1543,6 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1520,6 +1553,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1836,9 +1875,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1852,25 +1891,25 @@
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1886,19 +1925,19 @@
         <v>16</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1918,25 +1957,25 @@
         <v>17</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J4" s="9">
         <v>11</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1952,19 +1991,19 @@
         <v>18</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1984,19 +2023,19 @@
         <v>19</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -2016,19 +2055,19 @@
         <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J7" s="7">
         <v>6</v>
@@ -2048,19 +2087,19 @@
         <v>21</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -2080,19 +2119,19 @@
         <v>22</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="J9" s="7">
         <v>4</v>
@@ -2112,19 +2151,19 @@
         <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -2144,25 +2183,25 @@
         <v>24</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="J11" s="7">
         <v>8</v>
       </c>
       <c r="K11" s="14" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2178,19 +2217,19 @@
         <v>25</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -2210,19 +2249,19 @@
         <v>26</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -2242,19 +2281,19 @@
         <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="J14" s="9">
         <v>2</v>
@@ -2274,19 +2313,19 @@
         <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -2306,19 +2345,19 @@
         <v>29</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -2338,19 +2377,19 @@
         <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -2370,19 +2409,19 @@
         <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G18" s="10">
         <v>885012205080</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2402,19 +2441,19 @@
         <v>32</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -2434,19 +2473,19 @@
         <v>33</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2466,19 +2505,19 @@
         <v>34</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -2494,28 +2533,28 @@
       <c r="C22" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="D22" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="22" t="s">
-        <v>122</v>
-      </c>
-      <c r="F22" s="21" t="s">
-        <v>194</v>
-      </c>
-      <c r="G22" s="22" t="s">
-        <v>253</v>
-      </c>
-      <c r="H22" s="21" t="s">
-        <v>294</v>
-      </c>
-      <c r="I22" s="22" t="s">
-        <v>337</v>
-      </c>
-      <c r="J22" s="21">
+      <c r="E22" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="F22" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>252</v>
+      </c>
+      <c r="H22" s="20" t="s">
+        <v>293</v>
+      </c>
+      <c r="I22" s="21" t="s">
+        <v>336</v>
+      </c>
+      <c r="J22" s="20">
         <v>3</v>
       </c>
-      <c r="K22" s="21"/>
+      <c r="K22" s="20"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
@@ -2530,19 +2569,19 @@
         <v>36</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2562,19 +2601,19 @@
         <v>37</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2594,19 +2633,19 @@
         <v>38</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="J25" s="7">
         <v>2</v>
@@ -2626,19 +2665,19 @@
         <v>39</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="J26" s="9">
         <v>2</v>
@@ -2658,19 +2697,19 @@
         <v>40</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2690,19 +2729,19 @@
         <v>41</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J28" s="9">
         <v>4</v>
@@ -2722,19 +2761,19 @@
         <v>42</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2754,19 +2793,19 @@
         <v>43</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2786,19 +2825,19 @@
         <v>44</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J31" s="7">
         <v>2</v>
@@ -2818,19 +2857,19 @@
         <v>45</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J32" s="9">
         <v>8</v>
@@ -2850,19 +2889,19 @@
         <v>46</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2878,28 +2917,28 @@
       <c r="C34" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="D34" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="E34" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="F34" s="21" t="s">
-        <v>202</v>
-      </c>
-      <c r="G34" s="22" t="s">
-        <v>261</v>
-      </c>
-      <c r="H34" s="21" t="s">
-        <v>308</v>
-      </c>
-      <c r="I34" s="23" t="s">
-        <v>396</v>
-      </c>
-      <c r="J34" s="21">
-        <v>1</v>
-      </c>
-      <c r="K34" s="21"/>
+      <c r="E34" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="F34" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="G34" s="21" t="s">
+        <v>260</v>
+      </c>
+      <c r="H34" s="20" t="s">
+        <v>307</v>
+      </c>
+      <c r="I34" s="22" t="s">
+        <v>395</v>
+      </c>
+      <c r="J34" s="20">
+        <v>1</v>
+      </c>
+      <c r="K34" s="20"/>
     </row>
     <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
@@ -2910,28 +2949,28 @@
       <c r="C35" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D35" s="24" t="s">
+      <c r="D35" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E35" s="23" t="s">
-        <v>135</v>
-      </c>
-      <c r="F35" s="24" t="s">
-        <v>205</v>
-      </c>
-      <c r="G35" s="23" t="s">
-        <v>262</v>
-      </c>
-      <c r="H35" s="24" t="s">
-        <v>309</v>
-      </c>
-      <c r="I35" s="23" t="s">
-        <v>396</v>
-      </c>
-      <c r="J35" s="24">
-        <v>1</v>
-      </c>
-      <c r="K35" s="24"/>
+      <c r="E35" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="F35" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="G35" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="H35" s="23" t="s">
+        <v>308</v>
+      </c>
+      <c r="I35" s="22" t="s">
+        <v>395</v>
+      </c>
+      <c r="J35" s="23">
+        <v>1</v>
+      </c>
+      <c r="K35" s="23"/>
     </row>
     <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
@@ -2942,28 +2981,28 @@
       <c r="C36" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="D36" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="E36" s="22" t="s">
-        <v>136</v>
-      </c>
-      <c r="F36" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="G36" s="22" t="s">
-        <v>263</v>
-      </c>
-      <c r="H36" s="21" t="s">
-        <v>310</v>
-      </c>
-      <c r="I36" s="23" t="s">
-        <v>396</v>
-      </c>
-      <c r="J36" s="21">
-        <v>1</v>
-      </c>
-      <c r="K36" s="21"/>
+      <c r="E36" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="F36" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="G36" s="21" t="s">
+        <v>262</v>
+      </c>
+      <c r="H36" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="I36" s="22" t="s">
+        <v>395</v>
+      </c>
+      <c r="J36" s="20">
+        <v>1</v>
+      </c>
+      <c r="K36" s="20"/>
     </row>
     <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
@@ -2974,28 +3013,28 @@
       <c r="C37" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D37" s="24" t="s">
+      <c r="D37" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="E37" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="F37" s="24" t="s">
-        <v>207</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>264</v>
-      </c>
-      <c r="H37" s="24" t="s">
-        <v>311</v>
-      </c>
-      <c r="I37" s="23" t="s">
-        <v>396</v>
-      </c>
-      <c r="J37" s="24">
+      <c r="E37" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="F37" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="G37" s="22" t="s">
+        <v>263</v>
+      </c>
+      <c r="H37" s="23" t="s">
+        <v>310</v>
+      </c>
+      <c r="I37" s="22" t="s">
+        <v>395</v>
+      </c>
+      <c r="J37" s="23">
         <v>2</v>
       </c>
-      <c r="K37" s="24"/>
+      <c r="K37" s="23"/>
     </row>
     <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
@@ -3010,17 +3049,17 @@
         <v>51</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H38" s="9"/>
       <c r="I38" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
@@ -3040,17 +3079,17 @@
         <v>52</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="H39" s="7"/>
       <c r="I39" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -3070,17 +3109,17 @@
         <v>53</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="H40" s="9"/>
       <c r="I40" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J40" s="9">
         <v>2</v>
@@ -3100,19 +3139,19 @@
         <v>54</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J41" s="7">
         <v>1</v>
@@ -3128,28 +3167,28 @@
       <c r="C42" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="D42" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="E42" s="22" t="s">
-        <v>142</v>
-      </c>
-      <c r="F42" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="G42" s="22" t="s">
-        <v>266</v>
-      </c>
-      <c r="H42" s="21" t="s">
-        <v>313</v>
-      </c>
-      <c r="I42" s="23" t="s">
-        <v>396</v>
-      </c>
-      <c r="J42" s="21">
-        <v>1</v>
-      </c>
-      <c r="K42" s="21"/>
+      <c r="E42" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="F42" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="G42" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="H42" s="20" t="s">
+        <v>312</v>
+      </c>
+      <c r="I42" s="22" t="s">
+        <v>395</v>
+      </c>
+      <c r="J42" s="20">
+        <v>1</v>
+      </c>
+      <c r="K42" s="20"/>
     </row>
     <row r="43" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
@@ -3158,25 +3197,25 @@
         <v>41</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>56</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J43" s="7">
         <v>4</v>
@@ -3190,25 +3229,25 @@
         <v>42</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D44" s="9" t="s">
         <v>57</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="I44" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -3228,19 +3267,19 @@
         <v>58</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F45" s="7">
         <v>855115001</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J45" s="7">
         <v>2</v>
@@ -3254,25 +3293,25 @@
         <v>44</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D46" s="9" t="s">
         <v>59</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="I46" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J46" s="9">
         <v>1</v>
@@ -3286,25 +3325,25 @@
         <v>45</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D47" s="7" t="s">
         <v>60</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -3318,13 +3357,13 @@
         <v>46</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D48" s="9" t="s">
         <v>61</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F48" s="9">
         <v>533980367</v>
@@ -3333,10 +3372,10 @@
         <v>533980367</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="I48" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
@@ -3350,25 +3389,25 @@
         <v>47</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>62</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -3388,19 +3427,19 @@
         <v>63</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
@@ -3420,19 +3459,19 @@
         <v>64</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="J51" s="7">
         <v>1</v>
@@ -3452,19 +3491,19 @@
         <v>65</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="J52" s="9">
         <v>1</v>
@@ -3478,25 +3517,25 @@
         <v>51</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D53" s="7" t="s">
         <v>66</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J53" s="7">
         <v>1</v>
@@ -3516,7 +3555,7 @@
         <v>67</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F54" s="9">
         <v>2158</v>
@@ -3525,16 +3564,16 @@
         <v>2158</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J54" s="9">
         <v>2</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3544,25 +3583,25 @@
         <v>53</v>
       </c>
       <c r="C55" s="17" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D55" s="18" t="s">
         <v>68</v>
       </c>
       <c r="E55" s="19" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F55" s="18" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G55" s="18" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I55" s="19" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J55" s="18">
         <v>4</v>
@@ -3582,19 +3621,19 @@
         <v>69</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J56" s="9">
         <v>4</v>
@@ -3610,28 +3649,28 @@
       <c r="C57" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D57" s="24" t="s">
+      <c r="D57" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="E57" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="F57" s="24" t="s">
-        <v>223</v>
-      </c>
-      <c r="G57" s="23" t="s">
-        <v>268</v>
-      </c>
-      <c r="H57" s="24" t="s">
-        <v>322</v>
-      </c>
-      <c r="I57" s="23" t="s">
-        <v>396</v>
-      </c>
-      <c r="J57" s="24">
-        <v>1</v>
-      </c>
-      <c r="K57" s="24"/>
+      <c r="E57" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="F57" s="23" t="s">
+        <v>222</v>
+      </c>
+      <c r="G57" s="22" t="s">
+        <v>267</v>
+      </c>
+      <c r="H57" s="23" t="s">
+        <v>321</v>
+      </c>
+      <c r="I57" s="22" t="s">
+        <v>395</v>
+      </c>
+      <c r="J57" s="23">
+        <v>1</v>
+      </c>
+      <c r="K57" s="23"/>
     </row>
     <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
@@ -3646,19 +3685,19 @@
         <v>71</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I58" s="10" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="J58" s="9">
         <v>2</v>
@@ -3678,19 +3717,19 @@
         <v>72</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3710,19 +3749,19 @@
         <v>73</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="J60" s="9">
         <v>1</v>
@@ -3738,29 +3777,29 @@
       <c r="C61" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D61" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="F61" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="G61" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="H61" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="I61" s="8" t="s">
-        <v>364</v>
-      </c>
-      <c r="J61" s="7">
+      <c r="D61" s="23" t="s">
+        <v>403</v>
+      </c>
+      <c r="E61" s="22" t="s">
+        <v>160</v>
+      </c>
+      <c r="F61" s="23" t="s">
+        <v>223</v>
+      </c>
+      <c r="G61" s="22" t="s">
+        <v>271</v>
+      </c>
+      <c r="H61" s="23" t="s">
+        <v>294</v>
+      </c>
+      <c r="I61" s="22" t="s">
+        <v>363</v>
+      </c>
+      <c r="J61" s="23">
         <v>6</v>
       </c>
-      <c r="K61" s="24" t="s">
-        <v>402</v>
+      <c r="K61" s="25" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3773,22 +3812,22 @@
         <v>13</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J62" s="9">
         <v>4</v>
@@ -3805,22 +3844,22 @@
         <v>13</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="J63" s="7">
         <v>1</v>
@@ -3837,22 +3876,22 @@
         <v>13</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="J64" s="9">
         <v>2</v>
@@ -3869,22 +3908,22 @@
         <v>13</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="J65" s="7">
         <v>8</v>
@@ -3901,22 +3940,22 @@
         <v>13</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I66" s="10" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="J66" s="9">
         <v>1</v>
@@ -3933,22 +3972,22 @@
         <v>13</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3964,28 +4003,28 @@
       <c r="C68" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D68" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="E68" s="22" t="s">
-        <v>168</v>
-      </c>
-      <c r="F68" s="21" t="s">
-        <v>224</v>
-      </c>
-      <c r="G68" s="22" t="s">
-        <v>279</v>
-      </c>
-      <c r="H68" s="21" t="s">
-        <v>295</v>
-      </c>
-      <c r="I68" s="22" t="s">
-        <v>371</v>
-      </c>
-      <c r="J68" s="21">
-        <v>1</v>
-      </c>
-      <c r="K68" s="21"/>
+      <c r="D68" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="E68" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="F68" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="G68" s="21" t="s">
+        <v>278</v>
+      </c>
+      <c r="H68" s="20" t="s">
+        <v>294</v>
+      </c>
+      <c r="I68" s="21" t="s">
+        <v>370</v>
+      </c>
+      <c r="J68" s="20">
+        <v>1</v>
+      </c>
+      <c r="K68" s="20"/>
     </row>
     <row r="69" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
@@ -3997,22 +4036,22 @@
         <v>13</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="J69" s="7">
         <v>1</v>
@@ -4029,22 +4068,22 @@
         <v>13</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I70" s="10" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="J70" s="9">
         <v>2</v>
@@ -4061,22 +4100,22 @@
         <v>13</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="J71" s="7">
         <v>2</v>
@@ -4093,22 +4132,22 @@
         <v>13</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G72" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I72" s="10" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J72" s="9">
         <v>1</v>
@@ -4125,22 +4164,22 @@
         <v>13</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="J73" s="7">
         <v>2</v>
@@ -4157,22 +4196,22 @@
         <v>13</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J74" s="9">
         <v>1</v>
@@ -4189,22 +4228,22 @@
         <v>13</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="I75" s="8" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="J75" s="7">
         <v>1</v>
@@ -4221,22 +4260,22 @@
         <v>13</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G76" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="J76" s="9">
         <v>6</v>
@@ -4253,22 +4292,22 @@
         <v>13</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="I77" s="8" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="J77" s="7">
         <v>1</v>
@@ -4285,22 +4324,22 @@
         <v>13</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F78" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J78" s="9">
         <v>1</v>
@@ -4314,25 +4353,25 @@
         <v>77</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D79" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F79" s="7" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="I79" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J79" s="7">
         <v>1</v>
@@ -4346,13 +4385,13 @@
         <v>78</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F80" s="9">
         <v>750314597</v>
@@ -4361,10 +4400,10 @@
         <v>750314597</v>
       </c>
       <c r="H80" s="9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="I80" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J80" s="9">
         <v>1</v>
@@ -4381,22 +4420,22 @@
         <v>14</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F81" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G81" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H81" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I81" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J81" s="7">
         <v>1</v>
@@ -4413,22 +4452,22 @@
         <v>14</v>
       </c>
       <c r="D82" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F82" s="9" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G82" s="10" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H82" s="9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="I82" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J82" s="9">
         <v>1</v>
@@ -4445,22 +4484,22 @@
         <v>14</v>
       </c>
       <c r="D83" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F83" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H83" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="I83" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J83" s="7">
         <v>1</v>
@@ -4477,22 +4516,22 @@
         <v>14</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F84" s="9" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G84" s="10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H84" s="9" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I84" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J84" s="9">
         <v>1</v>
@@ -4509,22 +4548,22 @@
         <v>14</v>
       </c>
       <c r="D85" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F85" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G85" s="8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="H85" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I85" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J85" s="7">
         <v>1</v>
@@ -4541,22 +4580,22 @@
         <v>14</v>
       </c>
       <c r="D86" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F86" s="9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G86" s="10" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H86" s="9" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="I86" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J86" s="9">
         <v>1</v>
@@ -4573,20 +4612,20 @@
         <v>14</v>
       </c>
       <c r="D87" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F87" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G87" s="8" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="H87" s="7"/>
       <c r="I87" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J87" s="7">
         <v>1</v>
@@ -4603,20 +4642,20 @@
         <v>14</v>
       </c>
       <c r="D88" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F88" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G88" s="10" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="H88" s="9"/>
       <c r="I88" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J88" s="9">
         <v>1</v>
@@ -4633,22 +4672,22 @@
         <v>14</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F89" s="7" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G89" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H89" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I89" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J89" s="7">
         <v>1</v>
@@ -4661,25 +4700,25 @@
         <v>88</v>
       </c>
       <c r="C90" s="13" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D90" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="E90" s="8" t="s">
         <v>397</v>
       </c>
-      <c r="E90" s="8" t="s">
+      <c r="F90" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="F90" s="7" t="s">
+      <c r="G90" s="8" t="s">
         <v>399</v>
       </c>
-      <c r="G90" s="8" t="s">
+      <c r="H90" s="7" t="s">
         <v>400</v>
       </c>
-      <c r="H90" s="7" t="s">
-        <v>401</v>
-      </c>
       <c r="I90" s="8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J90" s="7">
         <v>1</v>

</xml_diff>

<commit_message>
#174 BOM highlight Update.
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Top_Board_v3.5/BOM/Client_BOM_LSS_Top_Board_v3.5.xlsx
+++ b/Design-Files/LSS_Top_Board_v3.5/BOM/Client_BOM_LSS_Top_Board_v3.5.xlsx
@@ -1230,11 +1230,15 @@
     <t>RTT03R330FTP</t>
   </si>
   <si>
+    <t xml:space="preserve">Addition Highlighted with RED </t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">R5, </t>
     </r>
     <r>
       <rPr>
+        <b/>
         <sz val="9"/>
         <color rgb="FFFF0000"/>
         <rFont val="Calibri"/>
@@ -1253,15 +1257,12 @@
       <t>, R32</t>
     </r>
   </si>
-  <si>
-    <t xml:space="preserve">Addition Highlighted with RED </t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1331,13 +1332,6 @@
     </font>
     <font>
       <strike/>
-      <sz val="9"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1555,11 +1549,11 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1875,9 +1869,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3778,7 +3772,7 @@
         <v>13</v>
       </c>
       <c r="D61" s="23" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E61" s="22" t="s">
         <v>160</v>
@@ -3798,8 +3792,8 @@
       <c r="J61" s="23">
         <v>6</v>
       </c>
-      <c r="K61" s="25" t="s">
-        <v>404</v>
+      <c r="K61" s="24" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>